<commit_message>
Record the GTM decision, and why it is a rejection
Raised as a way to protect Core Web Vitals, which is backwards: the
container is a loader, so adopting it means putting a new script in
front of every script already loading and calling that an optimisation.

The reason it is a rejection rather than a decline is the coverage
gates. Today a blocked GA4 request does not take down the pixel, and
neither touches PostHog — the failures are independent and partial.
Behind one container a single blocked request removes everything at
once, and that failure concentrates in privacy-conscious, mobile and
paid traffic, which is exactly the segment DOD-1 and DOD-3 count.

Also worth saying plainly in the document: tags are not what makes the
app entry page slow. Nothing loaded afterInteractive blocks the largest
contentful paint, so deferring analytics will not move 4,461ms. That is
a rendering problem and it is filed as C-12.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/internal/doc/nursia-analytics-sprint-tracker.xlsx
+++ b/internal/doc/nursia-analytics-sprint-tracker.xlsx
@@ -3857,7 +3857,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4286,8 +4286,66 @@
       </c>
       <c r="G16" s="5" t="inlineStr"/>
     </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Clarity tag (layout.tsx:138)</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Script strategy</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>afterInteractive</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="n"/>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Currently beforeInteractive — executes ahead of hydration. NUR-21</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr"/>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tag management</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>GTM</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="n"/>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Adds a loader in front of existing tags; one blocked container kills all measurement at once, threatening DOD-1 and DOD-3. See PRD</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="F5:F16">
+  <conditionalFormatting sqref="F5:F18">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Done"</formula>
     </cfRule>
@@ -4298,7 +4356,7 @@
       <formula>"In progress"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D5:D16">
+  <conditionalFormatting sqref="D5:D18">
     <cfRule type="cellIs" priority="4" operator="greaterThan" dxfId="1">
       <formula>4000</formula>
     </cfRule>
@@ -4308,8 +4366,8 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F5:F16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Not started,In progress,Blocked,In review,Done"</formula1>
+    <dataValidation sqref="F5:F18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Not started,In progress,Blocked,In review,Done,Decided"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
One workbook, two audiences, and it now says which is which
The book had grown to eleven sheets with nothing telling a reader which
of them were theirs. A growth lead opening the PostHog install spec
finds init options and concludes the whole thing is an engineering
document; an engineer opening Start here finds prose and skips the rest.
Both readings lose something the other needed.

So every sheet declares its audience in its subtitle, and the front
sheet gains a 'Who reads this' column that routes. Four sheets are for
everyone, four are engineering, one is the app team's, and two are
shared — the dashboard sheet most of all, since that is the deliverable
both sides are working toward.

Nothing was moved or split to achieve it. A second workbook for
non-engineers would drift from this one within a week, and the version
people quote would be whichever they happened to receive.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/internal/doc/nursia-analytics-sprint-tracker.xlsx
+++ b/internal/doc/nursia-analytics-sprint-tracker.xlsx
@@ -563,13 +563,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="76" customWidth="1" min="3" max="3"/>
-    <col width="62" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -582,7 +583,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Read this sheet first. Everything below is written for whoever funds the work, not only for whoever builds it.</t>
+          <t>Read this sheet first. The book serves two audiences: the 'Who reads this' column says which sheets are yours. Nothing here assumes you write code except where it says so.</t>
         </is>
       </c>
     </row>
@@ -603,6 +604,11 @@
           <t>Why it matters commercially</t>
         </is>
       </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Who reads this</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="44" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -621,6 +627,11 @@
           <t>Every pound of ad spend is currently unattributable to what it produced.</t>
         </is>
       </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Everyone</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="44" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
@@ -641,6 +652,11 @@
       <c r="D6" s="6" t="inlineStr">
         <is>
           <t>Smart Bidding is optimising toward an event that never happens. It is buying blind.</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Everyone</t>
         </is>
       </c>
     </row>
@@ -661,6 +677,11 @@
           <t>Meta cannot learn what a good customer looks like, so delivery stays broad and expensive.</t>
         </is>
       </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Everyone</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="44" customHeight="1">
       <c r="A8" s="4" t="inlineStr"/>
@@ -679,6 +700,11 @@
           <t>Nobody can answer: which channel brings people who actually study?</t>
         </is>
       </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Everyone</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="44" customHeight="1">
       <c r="A9" s="4" t="inlineStr"/>
@@ -697,6 +723,11 @@
           <t>A stolen session is a customer breach. Fix first, before anything else ships.</t>
         </is>
       </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Everyone</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="44" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
@@ -717,6 +748,11 @@
       <c r="D10" s="6" t="inlineStr">
         <is>
           <t>After it: budget moves on evidence rather than on click-through rate.</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Everyone</t>
         </is>
       </c>
     </row>
@@ -737,6 +773,11 @@
           <t>Deciding them takes an hour. Not deciding them costs the sprint.</t>
         </is>
       </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Everyone</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="44" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
@@ -757,6 +798,11 @@
       <c r="D12" s="6" t="inlineStr">
         <is>
           <t>Stops anyone declaring victory on instrumentation that does not work.</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Everyone</t>
         </is>
       </c>
     </row>
@@ -777,6 +823,11 @@
           <t>Read before sprint planning, not during.</t>
         </is>
       </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>Engineering + growth lead</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="44" customHeight="1">
       <c r="A14" s="4" t="inlineStr"/>
@@ -795,6 +846,11 @@
           <t>The 'Why it matters' column is the one to read if you do not write code.</t>
         </is>
       </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Everyone</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="44" customHeight="1">
       <c r="A15" s="4" t="inlineStr"/>
@@ -813,6 +869,11 @@
           <t>Shows at a glance which parts of the product are invisible.</t>
         </is>
       </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>Everyone</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="44" customHeight="1">
       <c r="A16" s="4" t="inlineStr"/>
@@ -831,6 +892,11 @@
           <t>Tick nothing you have not seen with your own eyes.</t>
         </is>
       </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="44" customHeight="1">
       <c r="A17" s="4" t="inlineStr"/>
@@ -849,6 +915,11 @@
           <t>The dashboard is the deliverable. Everything else exists to fill it.</t>
         </is>
       </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>Engineering / Growth</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="44" customHeight="1">
       <c r="A18" s="4" t="inlineStr"/>
@@ -867,6 +938,11 @@
           <t>A faster page converts better. The budget protects that while instrumentation is added.</t>
         </is>
       </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="44" customHeight="1">
       <c r="A19" s="4" t="inlineStr"/>
@@ -883,6 +959,11 @@
       <c r="D19" s="6" t="inlineStr">
         <is>
           <t>Twelve tickets depend on it. Confirm ownership before sprint start or the sprint cannot finish.</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>Engineering (external team)</t>
         </is>
       </c>
     </row>
@@ -919,7 +1000,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>GTM does not improve Core Web Vitals; a container loads tags rather than replacing them. But the autonomy case is real, and these are the ways to load it without paying full price. The final decision is engineering's — record it in G-07.</t>
+          <t>FOR ENGINEERING, DECIDED BY ENGINEERING. GTM does not improve Core Web Vitals; a container loads tags rather than replacing them. But the autonomy case is real, and these are the ways to load it without paying full price. The final decision is engineering's — record it in G-07.</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1320,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Not our repository. Twelve of twenty-four sprint tickets depend on this team. C-00 is a security fix and does not wait; C-01 to C-07 block activation and high-intent measurement entirely.</t>
+          <t>FOR THE APP TEAM. Not our repository. Twelve of the sprint tickets depend on them. C-00 is a security fix and does not wait; C-01 to C-07 block activation and high-intent measurement entirely.</t>
         </is>
       </c>
     </row>
@@ -1756,7 +1837,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>All six, or the sprint is not done. Each is measurable the day it is claimed, from a named surface. 'It looks right in DebugView' is not a gate.</t>
+          <t>FOR EVERYONE. All six, or the sprint is not done. Each is measurable the day it is claimed, from a named surface. 'It looks right in DebugView' is not a gate.</t>
         </is>
       </c>
     </row>
@@ -2080,7 +2161,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Each changes what gets built. Left undecided, each has a default that happens anyway — usually the worse one, chosen by whoever picks up the ticket first. Settled and NOT reopenable: dashboards are PostHog, Ads conversions stay on gtag, the six gates are the definition of done.</t>
+          <t>FOR ENGINEERING, WITH THE GROWTH LEAD. Each changes what gets built. Left undecided, each has a default that happens anyway — usually the worse one, chosen by whoever picks up the ticket first. Settled and NOT reopenable: dashboards are PostHog, Ads conversions stay on gtag, the six gates are the definition of done.</t>
         </is>
       </c>
     </row>
@@ -2482,7 +2563,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>60 points across 28 tickets. NUR-00 is security and does not wait for the sprint. NUR-01 to NUR-10 are P0 and stop money being spent blind; if the sprint is cut, it is cut after those. Read the last column if you do not write code.</t>
+          <t>FOR EVERYONE. 60 points across 28 tickets. NUR-00 is security and does not wait for the sprint. NUR-01 to NUR-10 are P0 and stop money being spent blind; if the sprint is cut, it is cut after those. Read the last column if you do not write code.</t>
         </is>
       </c>
     </row>
@@ -3955,7 +4036,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Nine product areas, each with its own owner and its own gap. Status mirrors the rails in the PRD.</t>
+          <t>FOR EVERYONE. Nine product areas, each with its own owner and its own gap. Status mirrors the rails in the PRD.</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4459,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tick each column only after seeing the event in PostHog, GA4 DebugView and Meta Test Events. Status reflects the estate as audited on 11 Sep 2026, not intent.</t>
+          <t>FOR ENGINEERING. Tick each column only after seeing the event in PostHog, GA4 DebugView and Meta Test Events. Status reflects the estate as audited on 11 Sep 2026, not intent.</t>
         </is>
       </c>
     </row>
@@ -5339,7 +5420,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>The single change that makes eight of the outcome rows answerable. The app already reports to project 595036; this side does not, so neither half can describe a whole customer. PH-03 and PH-10 are the two that fail quietly rather than loudly.</t>
+          <t>FOR ENGINEERING. The single change that makes eight of the outcome rows answerable. The app already reports to project 595036; this side does not, so neither half can describe a whole customer. PH-03 and PH-10 are the two that fail quietly rather than loudly.</t>
         </is>
       </c>
     </row>
@@ -5924,7 +6005,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Project NCLEX-Nursia (595036). Eleven tiles. Tiles 6 and 10 need no new instrumentation — build those first so the dashboard exists and carries real data while the rest fills in.</t>
+          <t>FOR GROWTH AND ENGINEERING. This is the deliverable. Project NCLEX-Nursia (595036). Eleven tiles; 6 and 10 need no new instrumentation — build those first so the dashboard exists and carries real data while the rest fills in.</t>
         </is>
       </c>
     </row>
@@ -6360,7 +6441,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Baseline p75 from PostHog $web_vitals, 30 days to 11 Sep 2026 (312 events, 17 people). Google thresholds: LCP good ≤2500ms / poor &gt;4000ms, CLS good ≤0.10, INP good ≤200ms.</t>
+          <t>FOR ENGINEERING. A faster page converts better, so this is a growth constraint enforced by engineers. Baseline p75 from PostHog $web_vitals, 30 days to 11 Sep 2026 (312 events, 17 people). Google thresholds: LCP good ≤2500ms / poor &gt;4000ms, CLS good ≤0.10, INP good ≤200ms.</t>
         </is>
       </c>
     </row>

</xml_diff>